<commit_message>
fix: harden health sync uploads
</commit_message>
<xml_diff>
--- a/docs/phase1/Honoured-V1.1-Progress-Tracker.xlsx
+++ b/docs/phase1/Honoured-V1.1-Progress-Tracker.xlsx
@@ -701,7 +701,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="45" t="inlineStr">
         <is>
-          <t>Progress, task status and open questions for the native iOS app and the web and database work it depends on. Last updated Oct 10; every status was checked against the code, the published web app and the live database.</t>
+          <t>Progress, task status and open questions for the native iOS app and the web and database work it depends on. Last updated Oct 11; every status was checked against the code, the published web app and the live database.</t>
         </is>
       </c>
       <c r="B2" s="46" t="n"/>
@@ -721,7 +721,7 @@
     <row r="5">
       <c r="A5" s="31" t="inlineStr">
         <is>
-          <t>WHERE THINGS STAND — Oct 10</t>
+          <t>WHERE THINGS STAND — Oct 11</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
     <row r="8" ht="64" customHeight="1">
       <c r="A8" s="47" t="inlineStr">
         <is>
-          <t>• V1.2 M3 (Word Tracker): the database part is live (applied Oct 10). The web part is built and tested (582/582) and waits for a publish; the iPhone part is committed (branch feat/m3-word-tracker, 18/18 Word Tracker tests) and waits for the merge and a new build. The review gaps are fixed: reads from any screen, words with combining marks, the cut-off reminder and Scrivener projects in the file picker. Left: the real-iPhone checks (Gate A and the 12 acceptance cases).</t>
+          <t>• V1.2 M3 (Word Tracker): built and live. The web app was published on Oct 10 and 11, the database holds the word scoring with the 24-hour starting-count window and the 30-minute sync grace window, and the iPhone code is on main. Checked end to end on the simulator against the live web app and database: all five formats, rename, move, delete and reconnect, reminders, and a read just after midnight that counted for the day before. Left: an iPhone build and the real-iPhone checks, starting with a Scrivener project from Dropbox (Gate A).</t>
         </is>
       </c>
       <c r="B8" s="48" t="n"/>
@@ -767,7 +767,7 @@
     <row r="9" ht="19" customHeight="1">
       <c r="A9" s="47" t="inlineStr">
         <is>
-          <t>• V1.2 M4 (Multi-Activity Calendar): not started. History already lists each Icon day on its own date.</t>
+          <t>• V1.2 M4 (Multi-Activity Calendar): built and live (published Oct 11). Each calendar day shows one band per result, and a tap opens a sheet with every result of the day, its time, and that day's journal notes and Voice of Change recordings. Checked on the simulator; a real-iPhone pass is left.</t>
         </is>
       </c>
       <c r="B9" s="48" t="n"/>
@@ -793,7 +793,7 @@
     <row r="11" ht="19" customHeight="1">
       <c r="A11" s="47" t="inlineStr">
         <is>
-          <t>• Needs attention: general Health data has not reached the server since Oct 7, while Icon readings still arrive (Open Item #20).</t>
+          <t>• Needs attention: the client's iPhone has not uploaded general Health data since Oct 2. Cause found on Oct 11: an upload batch too large for the server stays stuck at the head of the phone's queue. Fixed in the app; it takes effect with the next iPhone build (Open Item #20).</t>
         </is>
       </c>
       <c r="B11" s="48" t="n"/>
@@ -915,7 +915,7 @@
       </c>
       <c r="B17" s="32" t="inlineStr">
         <is>
-          <t>Oct 9 – 10</t>
+          <t>Oct 9 – 11</t>
         </is>
       </c>
       <c r="C17" s="32" t="n"/>
@@ -929,7 +929,7 @@
       </c>
       <c r="F17" s="35">
         <f>IF(COUNTIF('V1.2 Tasks'!B:B,"V1.2 M3")=0,0,COUNTIFS('V1.2 Tasks'!B:B,"V1.2 M3",'V1.2 Tasks'!H:H,"Done")/COUNTIF('V1.2 Tasks'!B:B,"V1.2 M3"))</f>
-        <v>0.14285714285714285</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="G17" s="50" t="inlineStr">
         <is>
@@ -945,7 +945,7 @@
       </c>
       <c r="B18" s="32" t="inlineStr">
         <is>
-          <t>Not scheduled</t>
+          <t>Oct 11</t>
         </is>
       </c>
       <c r="C18" s="32" t="n"/>
@@ -959,7 +959,7 @@
       </c>
       <c r="F18" s="35">
         <f>IF(COUNTIF('V1.2 Tasks'!B:B,"V1.2 M4")=0,0,COUNTIFS('V1.2 Tasks'!B:B,"V1.2 M4",'V1.2 Tasks'!H:H,"Done")/COUNTIF('V1.2 Tasks'!B:B,"V1.2 M4"))</f>
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="G18" s="50" t="inlineStr">
         <is>
@@ -985,7 +985,7 @@
       </c>
       <c r="F19" s="36">
         <f>IF(SUMPRODUCT(COUNTIF('V1.2 Tasks'!B:B,{"V1.2 M1","V1.2 M2","V1.2 M3","V1.2 M4"}))=0,0,SUMPRODUCT(COUNTIFS('V1.2 Tasks'!B:B,{"V1.2 M1","V1.2 M2","V1.2 M3","V1.2 M4"},'V1.2 Tasks'!H:H,"Done"))/SUMPRODUCT(COUNTIF('V1.2 Tasks'!B:B,{"V1.2 M1","V1.2 M2","V1.2 M3","V1.2 M4"})))</f>
-        <v>0.5666666666666667</v>
+        <v>0.8</v>
       </c>
       <c r="G19" s="26" t="n"/>
     </row>
@@ -1021,11 +1021,11 @@
       </c>
       <c r="B23" s="34">
         <f>COUNTIFS('V1.2 Tasks'!H:H,"Done",'V1.2 Tasks'!B:B,"V1.2 M*")</f>
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C23" s="34">
         <f>SUMIFS('V1.2 Tasks'!F:F,'V1.2 Tasks'!H:H,"Done",'V1.2 Tasks'!B:B,"V1.2 M*")</f>
-        <v>75</v>
+        <v>119</v>
       </c>
     </row>
     <row r="24">
@@ -1036,11 +1036,11 @@
       </c>
       <c r="B24" s="34">
         <f>COUNTIFS('V1.2 Tasks'!H:H,"In progress",'V1.2 Tasks'!B:B,"V1.2 M*")</f>
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C24" s="34">
         <f>SUMIFS('V1.2 Tasks'!F:F,'V1.2 Tasks'!H:H,"In progress",'V1.2 Tasks'!B:B,"V1.2 M*")</f>
-        <v>51</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25">
@@ -1051,11 +1051,11 @@
       </c>
       <c r="B25" s="34">
         <f>COUNTIFS('V1.2 Tasks'!H:H,"Not started",'V1.2 Tasks'!B:B,"V1.2 M*")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C25" s="34">
         <f>SUMIFS('V1.2 Tasks'!F:F,'V1.2 Tasks'!H:H,"Not started",'V1.2 Tasks'!B:B,"V1.2 M*")</f>
-        <v>27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -1098,7 +1098,7 @@
     <row r="30" ht="19" customHeight="1">
       <c r="A30" s="47" t="inlineStr">
         <is>
-          <t>• Publish the web app in Lovable and merge feat/m3-word-tracker into main, then ship an iPhone build with the Word Tracker.</t>
+          <t>• Ship an iPhone build from main: Word Tracker, sync grace window, password saving (X-07) and native session refresh (X-12).</t>
         </is>
       </c>
       <c r="B30" s="48" t="n"/>
@@ -1111,7 +1111,7 @@
     <row r="31" ht="19" customHeight="1">
       <c r="A31" s="47" t="inlineStr">
         <is>
-          <t>• Run the Word Tracker device checks: a Scrivener project from Dropbox or iCloud (Gate A), then the 12 acceptance cases (Gate D).</t>
+          <t>• Run the Word Tracker device checks (docs/phase2/M3-device-test-plan.vi.md): a Scrivener project from Dropbox first (Gate A), then the acceptance cases (Gate D).</t>
         </is>
       </c>
       <c r="B31" s="48" t="n"/>
@@ -1124,7 +1124,7 @@
     <row r="32" ht="19" customHeight="1">
       <c r="A32" s="47" t="inlineStr">
         <is>
-          <t>• Find out why general Health data stopped reaching the server on Oct 7 (Open Item #20).</t>
+          <t>• Install the next iPhone build on the client's iPhone and confirm its queued Health data arrives (Open Item #20).</t>
         </is>
       </c>
       <c r="B32" s="48" t="n"/>
@@ -1137,7 +1137,7 @@
     <row r="33" ht="34" customHeight="1">
       <c r="A33" s="47" t="inlineStr">
         <is>
-          <t>• Run the real-iPhone acceptance passes for M1 (Apple Watch and Garmin source) and M2 (evening card, fallback notification, sign-out).</t>
+          <t>• Run the real-iPhone acceptance passes for M1 (Apple Watch and Garmin source), M2 (evening card, fallback notification, sign-out) and M4 (calendar bands, day sheet, VoiceOver).</t>
         </is>
       </c>
       <c r="B33" s="48" t="n"/>
@@ -1150,7 +1150,7 @@
     <row r="34" ht="34" customHeight="1">
       <c r="A34" s="47" t="inlineStr">
         <is>
-          <t>• Client: publishing account, final App ID and APNs key (#14), Google client IDs (#15), and the decisions in Open Items #16–#18, #21 and #23–#25.</t>
+          <t>• Client: publishing account, final App ID and APNs key (#14), Google client IDs (#15), the decisions in Open Items #16–#18, #21, #23–#25 and #28, and a review of the two Word Tracker documents (#27).</t>
         </is>
       </c>
       <c r="B34" s="48" t="n"/>
@@ -1163,7 +1163,7 @@
     <row r="35" ht="19" customHeight="1">
       <c r="A35" s="47" t="inlineStr">
         <is>
-          <t>• Then TestFlight for the client and App Store submission (N-21, N-22), and start M4.</t>
+          <t>• Then TestFlight for the client and App Store submission (N-21, N-22).</t>
         </is>
       </c>
       <c r="B35" s="48" t="n"/>
@@ -1428,7 +1428,7 @@
       </c>
       <c r="B49" s="47" t="inlineStr">
         <is>
-          <t>The starting count is the last reading before the Icon day starts and the latest reading before the cut-off decides the day; the evening reminder is within 8 h before the cut-off (Sep 28). Scrivener stays in M3 unless a blocker is proven on a device.</t>
+          <t>The starting count is the last reading before the Icon day starts and the latest reading before the cut-off decides the day; the evening reminder is within 8 h before the cut-off (Sep 28). Scrivener stays in M3 unless a blocker is proven on a device. Refined on Oct 10–11 and awaiting confirmation: see Open Item #23.</t>
         </is>
       </c>
       <c r="C49" s="48" t="n"/>
@@ -2079,17 +2079,17 @@
       <c r="G10" s="29" t="n"/>
       <c r="H10" s="29" t="inlineStr">
         <is>
-          <t>Published web build 48b7a74 (Oct 7) carries every V1.1 web part and V1.2 M1 and M2. Icon card renewal before iOS's 8-hour limit and the Testament Timer for Icons (Oct 6); the client's Icon screen changes (Oct 6–7). A real iPhone has received server-started Icon cards since Oct 6, with a full cycle on Oct 9. The V1.2 M3 Word Tracker was built in code and tested on Oct 9–10 (iPhone 188/188, web 573/573, database 63/63); it is not live yet. Oct 10: the Word Tracker database change was applied to production; the review gaps were fixed (reads from any screen, combining marks, cut-off reminders, Scrivener in the file picker); the web part is built (not yet published) and the iPhone part is committed on a branch.</t>
+          <t>Published web build 48b7a74 (Oct 7) carries every V1.1 web part and V1.2 M1 and M2. Icon card renewal before iOS's 8-hour limit and the Testament Timer for Icons (Oct 6); the client's Icon screen changes (Oct 6–7). A real iPhone has received server-started Icon cards since Oct 6, with a full cycle on Oct 9. The V1.2 M3 Word Tracker was built in code and tested on Oct 9–10 (iPhone 188/188, web 573/573, database 63/63); it is not live yet. Oct 10: the Word Tracker database change was applied to production; the review gaps were fixed (reads from any screen, combining marks, cut-off reminders, Scrivener in the file picker); the web part is built (not yet published) and the iPhone part is committed on a branch. Oct 10–11: the Word Tracker went live (web published, three database changes, iPhone code on main) and passed end to end on the simulator, including the grace window across midnight; M4 (calendar bands and the day sheet) was built and published.</t>
         </is>
       </c>
       <c r="I10" s="29" t="inlineStr">
         <is>
-          <t>Publishing account and final App ID; Google client IDs for the iPhone app; the Word Tracker web publish and iPhone build. New: general Health data has not reached the server since Oct 7, while Icon readings still arrive.</t>
+          <t>Publishing account and final App ID; Google client IDs for the iPhone app; the Word Tracker web publish and iPhone build. The stalled Health upload (since Oct 2 on the client's iPhone) was traced and fixed in the app on Oct 11; it needs the next iPhone build.</t>
         </is>
       </c>
       <c r="J10" s="29" t="inlineStr">
         <is>
-          <t>Next: the Word Tracker rollout and fixes, the real-iPhone acceptance passes, and the Health upload investigation.</t>
+          <t>Next: an iPhone build, the real-iPhone acceptance passes (Word Tracker first, then M1, M2 and M4) and the Health upload investigation.</t>
         </is>
       </c>
     </row>
@@ -2106,12 +2106,12 @@
       </c>
       <c r="C11" s="28" t="inlineStr">
         <is>
-          <t>Word Tracker rollout and device acceptance</t>
+          <t>iPhone build and device acceptance</t>
         </is>
       </c>
       <c r="D11" s="28" t="inlineStr">
         <is>
-          <t>Publish the web and ship an iPhone build with the Word Tracker; Word Tracker device checks (Gate A, the 12 cases); real-iPhone passes for M1 and M2; Health upload investigation; client decisions (Open Items #14–#18, #21, #23–#25)</t>
+          <t>Ship an iPhone build from main; Word Tracker device checks (Gate A first, then Gate D); real-iPhone passes for M1, M2 and M4; Health upload investigation; client decisions (Open Items #14–#18, #21, #23–#25, #27, #28)</t>
         </is>
       </c>
       <c r="E11" s="28" t="inlineStr">
@@ -3288,12 +3288,12 @@
       </c>
       <c r="J24" s="29" t="inlineStr">
         <is>
-          <t>Sample .txt, .rtf, .rtfd, .docx and .scriv files generated in WordTrackerCoreTests.swift · format rules in docs/phase1/bridge.md · Pages feasibility note written (docs/phase2/Honoured V1.2 Pages Feasibility Note.md, Oct 10) · Gate A (a Scrivener project opened on a real iPhone) not run</t>
+          <t>Fixtures in all five formats (WordTrackerCoreTests) and real files picked through the Files picker on the simulator (Oct 10) · written findings and Pages feasibility note: 'Word Tracker Technical Findings' (Oct 11, with sources) · counting rules: 'Word Tracker Counting Rules' (Oct 10) · Gate A (a Scrivener project opened from Dropbox on a real iPhone) not run</t>
         </is>
       </c>
       <c r="K24" s="29" t="inlineStr">
         <is>
-          <t>The file-format rules are settled, the automated tests build sample files in all five formats, and the Pages note is written: Pages is not recommended for now because its file format is private and changes between versions. Still to do: open a real Scrivener project from Dropbox or iCloud on an iPhone (Gate A).</t>
+          <t>The file-format rules are settled and written up for the client, together with the Pages note: Pages counts look achievable on the iPhone, but Apple does not publish the format, so an adapter would need retesting after Pages updates. Still to do: open a real Scrivener project from Dropbox on an iPhone (Gate A).</t>
         </is>
       </c>
     </row>
@@ -3329,7 +3329,7 @@
       <c r="G25" s="28" t="n"/>
       <c r="H25" s="28" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I25" s="28" t="inlineStr">
@@ -3339,12 +3339,12 @@
       </c>
       <c r="J25" s="28" t="inlineStr">
         <is>
-          <t>Native commit 3a80410 (branch feat/m3-word-tracker): NativeBridge+WordTracker.swift, WordSourceBookmarkStore.swift · Keychain, this device only, per account and contract · bookmark created inside security-scoped access · stale bookmarks refreshed · reconnect keeps the source id · Scrivener package type declared in Info.plist · not yet run on a device</t>
+          <t>On main since Oct 10 (merge 1e18ab4) · simulator, Oct 10–11, real Files picker: rename, move, edit and relaunch keep the source; another account never sees it; a file in Recently Deleted counts as missing until recovered (ef13e5d) · scenarios word-tracker, word-tracker-check and word-tracker-delete (5cc53bd)</t>
         </is>
       </c>
       <c r="K25" s="28" t="inlineStr">
         <is>
-          <t>Choosing one document or project, remembering it securely on the phone and keeping each account's sources apart are built and committed. Waiting for the merge into main, an iPhone build and a device check (relaunch, rename, move, another account).</t>
+          <t>Choosing one document or project, remembering it securely on the phone and keeping each account's sources apart work on the simulator, including renamed, moved and recovered files. A deleted file now asks the writer to reconnect instead of counting the copy in Recently Deleted. The real-iPhone check is part of M3-07.</t>
         </is>
       </c>
     </row>
@@ -3380,7 +3380,7 @@
       <c r="G26" s="29" t="n"/>
       <c r="H26" s="29" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I26" s="29" t="inlineStr">
@@ -3390,12 +3390,12 @@
       </c>
       <c r="J26" s="29" t="inlineStr">
         <is>
-          <t>Native commit 3a80410: WordCount.swift (combining marks stay in their word, Chinese and Japanese characters count one each, 1,000 and 3.14 count once), WordSourceSupport.swift, WordDocumentReader.swift (.docx file and unzipped-XML size limits) · 18 Word Tracker tests pass, incl. the same 7-word text counting 7 in all five formats</t>
+          <t>WordTrackerCoreTests 20/20, whole native suite 196/196 (Oct 11) · the same chapter counted 49 in all five formats through the picker on the simulator · each read also reports when the counted content last changed, for the grace window (f341d84)</t>
         </is>
       </c>
       <c r="K26" s="29" t="inlineStr">
         <is>
-          <t>One counting rule for Word, TextEdit and Scrivener: the same text gives the same count in all five formats, also for Hindi, Arabic, Vietnamese, Chinese and Japanese text, and a damaged file returns an error instead of a wrong count. Committed; waiting for the merge into main and a comparison with real documents saved by each app.</t>
+          <t>One counting rule for Word, TextEdit and Scrivener gives the same count in all five formats, also for Vietnamese, Chinese, Japanese, Hindi and Arabic text, and a damaged file returns an error instead of a wrong count. The rule is written up in 'Word Tracker Counting Rules'.</t>
         </is>
       </c>
     </row>
@@ -3431,7 +3431,7 @@
       <c r="G27" s="28" t="n"/>
       <c r="H27" s="28" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I27" s="28" t="inlineStr">
@@ -3441,12 +3441,12 @@
       </c>
       <c r="J27" s="28" t="inlineStr">
         <is>
-          <t>Native 3a80410: SELECT / GET / READ / REMOVE_WORD_SOURCE, CLEAR_WORD_SOURCES and SET_WORD_REMINDERS (quiet reminder 30 minutes before the cut-off) · web Lovable bfdbbfa: automatic reads from any screen, on return to the app and every 10 minutes; reminder list synced to the phone · web not yet published</t>
+          <t>Live with the published web app (Lovable b52852e Oct 10, 68d8563 Oct 11): reads on start, on return, every 10 minutes, on Check now and right after signing; Reconnect shows 'Reconnect the same source to keep this Icon.'; the phone holds a reminder 30 minutes before each pending cut-off (checked on the simulator) · bridge: only ids, kind, count, read and change times and a random revision cross (docs/phase1/bridge.md)</t>
         </is>
       </c>
       <c r="K27" s="28" t="inlineStr">
         <is>
-          <t>Only counts and anonymous IDs pass between the app and the web page. The count is read when the app opens on any screen, when it returns to the foreground, every 10 minutes while open and on 'Check now', and the phone reminds the writer 30 minutes before the cut-off. Waiting for the web publish and an iPhone build.</t>
+          <t>Only counts, times and anonymous IDs pass between the app and the web page. The count is read when the app opens, when it returns, every 10 minutes, on 'Check now' and right after signing, and the phone reminds the writer 30 minutes before the cut-off.</t>
         </is>
       </c>
     </row>
@@ -3492,12 +3492,12 @@
       </c>
       <c r="J28" s="29" t="inlineStr">
         <is>
-          <t>Applied to production on Oct 10 as migration 0001_word_tracker_v1 (Lovable 488c619) · the four live functions match the tested SQL exactly (63/63 behavioural checks) · row-level security on word_source_readings, no client access · the 15-minute expiry job keeps succeeding after the change · undo script ready</t>
+          <t>Applied to production on Oct 10 as migration 0001_word_tracker_v1 (Lovable 488c619) · the four live functions match the tested SQL exactly (63/63 behavioural checks) · row-level security on word_source_readings, no client access · the 15-minute expiry job keeps succeeding after the change · undo script ready · Oct 10: 0002_word_baseline_window (a stored reading is the starting count only within the 24 hours before the day) · Oct 11: 0003_word_grace_window (a read up to 30 minutes after the cut-off counts when the document last changed before it; exact starting count when unchanged since midnight); both checked in the live database</t>
         </is>
       </c>
       <c r="K28" s="29" t="inlineStr">
         <is>
-          <t>The database change for word Icons is live: word columns, the reading log, the scoring function and the 24-hour rule for days nobody could verify. Health and self-report Icons are unchanged. The starting-count rule and the target range can still be adjusted with a follow-up change if the client asks (Open Items #23, #24).</t>
+          <t>The database change for word Icons is live, with two follow-ups on Oct 10–11: the starting count only comes from a reading in the 24 hours before the day, and the 30-minute sync grace window from the scope. Tested across a real midnight: a read at 00:02 counted for the day before. The starting-count rule awaits the client's confirmation (Open Item #23).</t>
         </is>
       </c>
     </row>
@@ -3533,7 +3533,7 @@
       <c r="G29" s="28" t="n"/>
       <c r="H29" s="28" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I29" s="28" t="inlineStr">
@@ -3543,12 +3543,12 @@
       </c>
       <c r="J29" s="28" t="inlineStr">
         <is>
-          <t>Lovable eb40dcf → bfdbbfa (Oct 10): words unit, writing-source row, signing gate, progress block, Reconnect, app-level reads and reminders, source cleanup, the scope's privacy wording · 582/582 web tests, typecheck and build pass · not yet published (the live site is still 48b7a74)</t>
+          <t>Published Oct 10 and 11 · simulator against the live database: signed a 100-word Icon, start 49 → +110 HONOURED, Replace before signing, Reconnect keeps the locked source id · fixes: progress shows without REFRESH, the source error clears once a source is chosen, the missing-source message names Reconnect (b52852e) · web tests 622/622 (Oct 11)</t>
         </is>
       </c>
       <c r="K29" s="28" t="inlineStr">
         <is>
-          <t>Writing can be committed in words: a word Icon needs its writing source before signing and then shows the starting count, the current count and the net words. Built and tested; it goes live with the next web publish and needs the new iPhone build to be used.</t>
+          <t>Writing can be committed in words, and the Icon shows the starting count, the current count and the net words right after signing. Checked end to end on the simulator against the live database.</t>
         </is>
       </c>
     </row>
@@ -3594,12 +3594,12 @@
       </c>
       <c r="J30" s="29" t="inlineStr">
         <is>
-          <t>Automated: 18/18 Word Tracker tests with the whole app compiled (the full native suite last passed 188/188 before the final fixes), web 582/582, database 63/63 plus the live checks · not done: the real-iPhone run of the 12 acceptance cases (Gate D) and the joint run of the new iPhone build, the published web and the live database (Gate C)</t>
+          <t>Simulator end to end with the live web app and database, Oct 10–11, including the grace window across a real midnight · device test plan: docs/phase2/M3-device-test-plan.vi.md · screenshots and scenario logs: outputs/v12-m3-m4-20261011 · not done: the real-iPhone run (Gate A Scrivener from Dropbox, Gate D)</t>
         </is>
       </c>
       <c r="K30" s="29" t="inlineStr">
         <is>
-          <t>Automated checks pass for the iPhone, web and database parts, and the database part is live. The real-iPhone acceptance run of all 12 cases (including Scrivener and account switching) follows the web publish and the new iPhone build.</t>
+          <t>Everything that can be checked without a real iPhone passes. Left: the real-iPhone pass with iCloud Drive, Dropbox and OneDrive files, Scrivener from Dropbox first.</t>
         </is>
       </c>
     </row>
@@ -3635,7 +3635,7 @@
       <c r="G31" s="28" t="n"/>
       <c r="H31" s="28" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I31" s="28" t="inlineStr">
@@ -3645,12 +3645,12 @@
       </c>
       <c r="J31" s="28" t="inlineStr">
         <is>
-          <t>Searched both repositories and the Lovable history: no M4 work beyond the estimate · the schema already allows several contracts per person per day · head start: history-entries.ts lists each Icon day separately (Lovable 499d0dd, Oct 5)</t>
+          <t>Schema already allows several contracts per person per day (checked Oct 11: no per-day unique key; live data has days with up to 9 contracts) · Lovable 6c0fee7 (Oct 11): resultsByDay and journalEntriesByDay in history-entries.ts; a regular contract sits on the date it was signed · no migration</t>
         </is>
       </c>
       <c r="K31" s="28" t="inlineStr">
         <is>
-          <t>Not started. The database already allows several contracts per person on the same day, and since Oct 5 History lists each Icon day as its own entry, which gives this task a head start.</t>
+          <t>Every result of a day is kept for that day; nothing is merged or dropped. A regular contract now sits on the date it was signed (it used to be the date it ended), so a contract that runs past midnight stays on its day (Open Item #28).</t>
         </is>
       </c>
     </row>
@@ -3686,7 +3686,7 @@
       <c r="G32" s="29" t="n"/>
       <c r="H32" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I32" s="29" t="inlineStr">
@@ -3696,12 +3696,12 @@
       </c>
       <c r="J32" s="29" t="inlineStr">
         <is>
-          <t>History.tsx at Lovable 774afec: one colour per date (its newest result); each cell is already one button; no band component</t>
+          <t>Lovable 6c0fee7, published Oct 11: HistoryDayCell (equal-height full-width bands in time order, white centred day number with a shadow, one button per day, the filter dims bands that do not match, spoken label); shared result colours in result-colours.ts, also used by the Icon marks · simulator: Oct 10 shows six bands</t>
         </is>
       </c>
       <c r="K32" s="29" t="inlineStr">
         <is>
-          <t>Not started. Today each date shows one colour (its latest result), and tapping a date already selects it. The coloured bands for several results and the white centred day number are still to build.</t>
+          <t>Each date shows one band per result in green, red or amber, with the day number in white on top, and the whole day is one tap target. The colours now match the Icon marks.</t>
         </is>
       </c>
     </row>
@@ -3737,7 +3737,7 @@
       <c r="G33" s="28" t="n"/>
       <c r="H33" s="28" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I33" s="28" t="inlineStr">
@@ -3747,12 +3747,12 @@
       </c>
       <c r="J33" s="28" t="inlineStr">
         <is>
-          <t>History.tsx at Lovable 774afec: an inline panel for one entry; no result time, journal text or recording playback; no day-sheet component</t>
+          <t>Lovable 6c0fee7 + 0371495, published Oct 11: HistoryDaySheet (swipe, close button, Escape, backdrop, focus) listing every result with activity, target, result, time, session, Health or word result and the reason; journal entries with Voice of Change playback and 'Recording unavailable' · simulator: six results on Oct 10; a note and a 10-second recording played on Oct 11</t>
         </is>
       </c>
       <c r="K33" s="28" t="inlineStr">
         <is>
-          <t>Not started. Tapping a date today opens a small panel for one result and lists that day's results below it. The full day sheet with time, journal entry and Voice of Change is still to build.</t>
+          <t>Tapping a date opens a sheet with every result of that day and its time, followed by that day's journal notes and Voice of Change recordings, which play in place.</t>
         </is>
       </c>
     </row>
@@ -3788,7 +3788,7 @@
       <c r="G34" s="29" t="n"/>
       <c r="H34" s="29" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="I34" s="29" t="inlineStr">
@@ -3798,12 +3798,12 @@
       </c>
       <c r="J34" s="29" t="inlineStr">
         <is>
-          <t>No M4 tests or QA notes yet</t>
+          <t>Web tests 622/622 in four time zones (tests/history-calendar.test.ts, history-entries.test.ts) · simulator pass on Oct 11; one wording fix (0371495) · not done: a real iPhone (legibility, swipe, VoiceOver, a busy month)</t>
         </is>
       </c>
       <c r="K34" s="29" t="inlineStr">
         <is>
-          <t>Not started; follows the calendar and day sheet work.</t>
+          <t>Automated tests and the simulator pass, and the one issue found was fixed. A real-iPhone pass is left.</t>
         </is>
       </c>
     </row>
@@ -4141,12 +4141,12 @@
       </c>
       <c r="J41" s="28" t="inlineStr">
         <is>
-          <t>Web: Lovable 768dd27 (Oct 3), 203c1ef (Oct 4), 48b7a74 (Oct 7: SAVE_WEB_CREDENTIAL and the apple-app-site-association file) · native: no SAVE_WEB_CREDENTIAL handler or Associated Domains entitlement yet; the file lists only the test App ID</t>
+          <t>Web: Lovable 768dd27 (Oct 3), 203c1ef (Oct 4), 48b7a74 (Oct 7) · native: 2d925b7 on main since Oct 10 (SAVE_WEB_CREDENTIAL, webcredentials associated domain) · the apple-app-site-association file lists only the test App ID · no device check yet</t>
         </is>
       </c>
       <c r="K41" s="28" t="inlineStr">
         <is>
-          <t>The web side is live and asks the iPhone to save the login to Passwords after sign-in or sign-up. The app still needs the matching native handler and Associated Domains for the final App ID, so the save prompt does not appear in the app yet.</t>
+          <t>Both sides are built: the web page asks the iPhone to save the login and the app shows the system prompt. Left: a device check, and the final App ID in the web app's association file before release.</t>
         </is>
       </c>
     </row>
@@ -4386,12 +4386,12 @@
       </c>
       <c r="J46" s="29" t="inlineStr">
         <is>
-          <t>Web: Lovable c191672 + 5b7b39f (Oct 7): native-session-refresh.ts, tests · native: no REFRESH_AUTH_SESSION handler or sessionRefresh capability yet</t>
+          <t>Web: Lovable c191672 + 5b7b39f (Oct 7) · native: 16f9f3f on main since Oct 10 (REFRESH_AUTH_SESSION, sessionRefresh capability) · no device check yet</t>
         </is>
       </c>
       <c r="K46" s="29" t="inlineStr">
         <is>
-          <t>The web side is live and waits for the iPhone app to take over session refresh. The native part is not built yet, so for now the page keeps refreshing the session itself, as before.</t>
+          <t>Both sides are built: the iPhone app now refreshes the web sign-in session. Left: a device check with an expired session.</t>
         </is>
       </c>
     </row>
@@ -5727,12 +5727,12 @@
       </c>
       <c r="J27" s="28" t="inlineStr">
         <is>
-          <t>Fixes: f6e9891, 5b84381, 7aaf06d, b33c764, 59055e8, 5a1dd1e; Lovable e6e07b5 · open: general Health uploads stalled (Open Item #20); Settings shows version 1.0.0 while the app is 1.0.5</t>
+          <t>Fixes: f6e9891, 5b84381, 7aaf06d, b33c764, 59055e8, 5a1dd1e; Lovable e6e07b5 · Oct 11: the stalled Health upload is fixed in the app (uploads split into small parts, refused rows isolated; Open Item #20), waiting for an iPhone build; Settings shows version 1.0.0 while the app is 1.0.5</t>
         </is>
       </c>
       <c r="K27" s="28" t="inlineStr">
         <is>
-          <t>Bugs found so far in testing have been fixed in the app and on the web. Known issues before release: general Health uploads have stalled (Icon readings still arrive), and Settings still shows version 1.0.0.</t>
+          <t>Bugs found so far in testing have been fixed in the app and on the web. Known issues before release: the stalled Health upload is fixed in the app and waits for the next iPhone build, and Settings still shows version 1.0.0.</t>
         </is>
       </c>
     </row>
@@ -6294,7 +6294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.005000114440918" customWidth="1" style="12" min="1" max="1"/>
@@ -7049,10 +7049,14 @@
       </c>
       <c r="F24" s="29" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="G24" s="29" t="n"/>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="G24" s="29" t="inlineStr">
+        <is>
+          <t>Oct 11: the client's iPhone (release build, Garmin heart-rate data) still sends Icon readings but no Health upload has arrived since Oct 2. The phone sends each collection as one request; dense watch data makes a batch of tens of thousands of samples, and the server's gateway drops any request over about 16 MB without answering (measured). The app kept retrying that batch forever, and every later batch waited behind it. The server and the session are fine (an upload from the simulator returned 200). Fixed in the app: uploads go in parts of at most 2,000 samples (about 0.5 MB), a queue already stuck on a phone is split when the app starts, and rows the server refuses are isolated and dropped instead of blocking the queue. Checked on the simulator: a stuck 75,000-sample batch uploaded in about 20 s. Takes effect when the new build is installed on the client's iPhone.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="76.5" customHeight="1">
       <c r="A25" s="8" t="n">
@@ -7147,7 +7151,7 @@
       </c>
       <c r="G27" s="28" t="inlineStr">
         <is>
-          <t>Built this way and live since Oct 10; it can be changed with a follow-up database change.</t>
+          <t>Updated Oct 10–11, live, waiting for your confirmation: the starting count is the last reading in the 24 hours before the Icon day starts; when the document has not changed since midnight, the day's first reading is the exact start; otherwise the day's first reading. Words written between the last check and midnight therefore count toward the next Icon day, never twice. A read up to 30 minutes after the cut-off counts when the document last changed before it.</t>
         </is>
       </c>
     </row>
@@ -7253,6 +7257,76 @@
       <c r="G30" s="29" t="inlineStr">
         <is>
           <t>Applied Oct 10 as migration 0001_word_tracker_v1. The live functions match the tested SQL, row-level security and grants were checked, and the expiry job runs normally. The undo script is ready.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="76.5" customHeight="1">
+      <c r="A31" s="22" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="29" t="inlineStr">
+        <is>
+          <t>Word Tracker: review the counting rules and the technical findings (Scrivener status, Pages note)</t>
+        </is>
+      </c>
+      <c r="C31" s="29" t="inlineStr">
+        <is>
+          <t>The scope asks for written findings and a Pages note before acceptance, and the counting rule explains why a count can differ slightly from Word's own.</t>
+        </is>
+      </c>
+      <c r="D31" s="29" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="E31" s="29" t="inlineStr">
+        <is>
+          <t>Week 6</t>
+        </is>
+      </c>
+      <c r="F31" s="29" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G31" s="29" t="inlineStr">
+        <is>
+          <t>Written Oct 10–11: 'Word Tracker Counting Rules' (https://claude.ai/artifact/NEwgWzgy5C9irPcNGCTCf7) and 'Word Tracker Technical Findings' (https://claude.ai/artifact/V9s8uKkEPc2Up4y2E5fQJG).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="76.5" customHeight="1">
+      <c r="A32" s="22" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="29" t="inlineStr">
+        <is>
+          <t>History: show a regular contract on the date it was signed?</t>
+        </is>
+      </c>
+      <c r="C32" s="29" t="inlineStr">
+        <is>
+          <t>M4 puts every result on its own day. A regular contract used to sit on the date it ended, so one that ran past midnight showed on the next day.</t>
+        </is>
+      </c>
+      <c r="D32" s="29" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="E32" s="29" t="inlineStr">
+        <is>
+          <t>Before M4 sign-off</t>
+        </is>
+      </c>
+      <c r="F32" s="29" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G32" s="29" t="inlineStr">
+        <is>
+          <t>Built this way and live since Oct 11; it can be switched back with a small web change.</t>
         </is>
       </c>
     </row>
@@ -7602,76 +7676,256 @@
       </c>
     </row>
     <row r="14" ht="120" customFormat="1" customHeight="1" s="5">
-      <c r="A14" s="29" t="n"/>
-      <c r="B14" s="29" t="n"/>
-      <c r="C14" s="29" t="n"/>
-      <c r="D14" s="29" t="n"/>
-      <c r="E14" s="29" t="n"/>
-      <c r="F14" s="29" t="n"/>
+      <c r="A14" s="28" t="inlineStr">
+        <is>
+          <t>Oct 10</t>
+        </is>
+      </c>
+      <c r="B14" s="28" t="inlineStr">
+        <is>
+          <t>Week 5</t>
+        </is>
+      </c>
+      <c r="C14" s="28" t="inlineStr">
+        <is>
+          <t>M3-01</t>
+        </is>
+      </c>
+      <c r="D14" s="28" t="inlineStr">
+        <is>
+          <t>Files picker in the Debug test harness offering all five formats, with the Scrivener project as one item</t>
+        </is>
+      </c>
+      <c r="E14" s="28" t="n"/>
+      <c r="F14" s="28" t="inlineStr">
+        <is>
+          <t>outputs/v12-m3-m4-20261011/m3-picker-five-formats.png (scenario logs alongside)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="120" customFormat="1" customHeight="1" s="5">
-      <c r="A15" s="28" t="n"/>
-      <c r="B15" s="28" t="n"/>
-      <c r="C15" s="28" t="n"/>
-      <c r="D15" s="28" t="n"/>
+      <c r="A15" s="28" t="inlineStr">
+        <is>
+          <t>Oct 10</t>
+        </is>
+      </c>
+      <c r="B15" s="28" t="inlineStr">
+        <is>
+          <t>Week 5</t>
+        </is>
+      </c>
+      <c r="C15" s="28" t="inlineStr">
+        <is>
+          <t>M3-06</t>
+        </is>
+      </c>
+      <c r="D15" s="28" t="inlineStr">
+        <is>
+          <t>Word Icon on the live web app after choosing its source: only 'Word document' is shown, never a file name</t>
+        </is>
+      </c>
       <c r="E15" s="28" t="n"/>
-      <c r="F15" s="28" t="n"/>
+      <c r="F15" s="28" t="inlineStr">
+        <is>
+          <t>outputs/v12-m3-m4-20261011/m3-word-source-chosen.png</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="120" customFormat="1" customHeight="1" s="5">
-      <c r="A16" s="29" t="n"/>
-      <c r="B16" s="29" t="n"/>
-      <c r="C16" s="29" t="n"/>
-      <c r="D16" s="29" t="n"/>
-      <c r="E16" s="29" t="n"/>
-      <c r="F16" s="29" t="n"/>
+      <c r="A16" s="28" t="inlineStr">
+        <is>
+          <t>Oct 10</t>
+        </is>
+      </c>
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>Week 5</t>
+        </is>
+      </c>
+      <c r="C16" s="28" t="inlineStr">
+        <is>
+          <t>M3-06</t>
+        </is>
+      </c>
+      <c r="D16" s="28" t="inlineStr">
+        <is>
+          <t>Word Icon day HONOURED: Start 49 · Now 159 · +110 of 100 words</t>
+        </is>
+      </c>
+      <c r="E16" s="28" t="n"/>
+      <c r="F16" s="28" t="inlineStr">
+        <is>
+          <t>outputs/v12-m3-m4-20261011/m3-word-icon-honoured.png</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="120" customFormat="1" customHeight="1" s="5">
-      <c r="A17" s="28" t="n"/>
-      <c r="B17" s="28" t="n"/>
-      <c r="C17" s="28" t="n"/>
-      <c r="D17" s="28" t="n"/>
+      <c r="A17" s="28" t="inlineStr">
+        <is>
+          <t>Oct 11</t>
+        </is>
+      </c>
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>Week 5</t>
+        </is>
+      </c>
+      <c r="C17" s="28" t="inlineStr">
+        <is>
+          <t>M3-04</t>
+        </is>
+      </c>
+      <c r="D17" s="28" t="inlineStr">
+        <is>
+          <t>Source moved to Recently Deleted: Reconnect with 'Reconnect the same source to keep this Icon.'</t>
+        </is>
+      </c>
       <c r="E17" s="28" t="n"/>
-      <c r="F17" s="28" t="n"/>
+      <c r="F17" s="28" t="inlineStr">
+        <is>
+          <t>outputs/v12-m3-m4-20261011/m3-reconnect-message.png</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="120" customFormat="1" customHeight="1" s="5">
-      <c r="A18" s="29" t="n"/>
-      <c r="B18" s="29" t="n"/>
-      <c r="C18" s="29" t="n"/>
-      <c r="D18" s="29" t="n"/>
-      <c r="E18" s="29" t="n"/>
-      <c r="F18" s="29" t="n"/>
+      <c r="A18" s="28" t="inlineStr">
+        <is>
+          <t>Oct 10</t>
+        </is>
+      </c>
+      <c r="B18" s="28" t="inlineStr">
+        <is>
+          <t>Week 5</t>
+        </is>
+      </c>
+      <c r="C18" s="28" t="inlineStr">
+        <is>
+          <t>M3-04</t>
+        </is>
+      </c>
+      <c r="D18" s="28" t="inlineStr">
+        <is>
+          <t>Quiet word reminder before the cut-off on the Home Screen (from the test harness)</t>
+        </is>
+      </c>
+      <c r="E18" s="28" t="n"/>
+      <c r="F18" s="28" t="inlineStr">
+        <is>
+          <t>outputs/v12-m3-m4-20261011/m3-cutoff-reminder.png</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="120" customFormat="1" customHeight="1" s="5">
-      <c r="A19" s="28" t="n"/>
-      <c r="B19" s="28" t="n"/>
-      <c r="C19" s="28" t="n"/>
-      <c r="D19" s="28" t="n"/>
+      <c r="A19" s="28" t="inlineStr">
+        <is>
+          <t>Oct 11</t>
+        </is>
+      </c>
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>Week 5</t>
+        </is>
+      </c>
+      <c r="C19" s="28" t="inlineStr">
+        <is>
+          <t>M4-02</t>
+        </is>
+      </c>
+      <c r="D19" s="28" t="inlineStr">
+        <is>
+          <t>History calendar: six equal bands on Oct 10, one per result, with the white day number</t>
+        </is>
+      </c>
       <c r="E19" s="28" t="n"/>
-      <c r="F19" s="28" t="n"/>
+      <c r="F19" s="28" t="inlineStr">
+        <is>
+          <t>outputs/v12-m3-m4-20261011/m4-calendar-bands.png</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="120" customFormat="1" customHeight="1" s="5">
-      <c r="A20" s="29" t="n"/>
-      <c r="B20" s="29" t="n"/>
-      <c r="C20" s="29" t="n"/>
-      <c r="D20" s="29" t="n"/>
-      <c r="E20" s="29" t="n"/>
-      <c r="F20" s="29" t="n"/>
+      <c r="A20" s="28" t="inlineStr">
+        <is>
+          <t>Oct 11</t>
+        </is>
+      </c>
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>Week 5</t>
+        </is>
+      </c>
+      <c r="C20" s="28" t="inlineStr">
+        <is>
+          <t>M4-03</t>
+        </is>
+      </c>
+      <c r="D20" s="28" t="inlineStr">
+        <is>
+          <t>Day sheet for Oct 10: every result with its time, session and word progress</t>
+        </is>
+      </c>
+      <c r="E20" s="28" t="n"/>
+      <c r="F20" s="28" t="inlineStr">
+        <is>
+          <t>outputs/v12-m3-m4-20261011/m4-day-sheet.png</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="120" customFormat="1" customHeight="1" s="5">
-      <c r="A21" s="28" t="n"/>
-      <c r="B21" s="28" t="n"/>
-      <c r="C21" s="28" t="n"/>
-      <c r="D21" s="28" t="n"/>
+      <c r="A21" s="28" t="inlineStr">
+        <is>
+          <t>Oct 11</t>
+        </is>
+      </c>
+      <c r="B21" s="28" t="inlineStr">
+        <is>
+          <t>Week 5</t>
+        </is>
+      </c>
+      <c r="C21" s="28" t="inlineStr">
+        <is>
+          <t>M4-03</t>
+        </is>
+      </c>
+      <c r="D21" s="28" t="inlineStr">
+        <is>
+          <t>Day sheet with a journal note and a Voice of Change recording that plays in place</t>
+        </is>
+      </c>
       <c r="E21" s="28" t="n"/>
-      <c r="F21" s="28" t="n"/>
+      <c r="F21" s="28" t="inlineStr">
+        <is>
+          <t>outputs/v12-m3-m4-20261011/m4-day-sheet-journal-voice.png</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="120" customFormat="1" customHeight="1" s="5">
-      <c r="A22" s="29" t="n"/>
-      <c r="B22" s="29" t="n"/>
-      <c r="C22" s="29" t="n"/>
-      <c r="D22" s="29" t="n"/>
-      <c r="E22" s="29" t="n"/>
-      <c r="F22" s="29" t="n"/>
+      <c r="A22" s="28" t="inlineStr">
+        <is>
+          <t>Oct 11</t>
+        </is>
+      </c>
+      <c r="B22" s="28" t="inlineStr">
+        <is>
+          <t>Week 5</t>
+        </is>
+      </c>
+      <c r="C22" s="28" t="inlineStr">
+        <is>
+          <t>M4-02</t>
+        </is>
+      </c>
+      <c r="D22" s="28" t="inlineStr">
+        <is>
+          <t>HONOURED filter: the broken day is hidden and amended bands are dimmed</t>
+        </is>
+      </c>
+      <c r="E22" s="28" t="n"/>
+      <c r="F22" s="28" t="inlineStr">
+        <is>
+          <t>outputs/v12-m3-m4-20261011/m4-filter-honoured.png</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="120" customFormat="1" customHeight="1" s="5">
       <c r="A23" s="28" t="n"/>

</xml_diff>